<commit_message>
Cambios en vista de logs, y tambien trasnferencia masiva
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Junio_PRE_SAP_TOOLS\pre_sap_cajas\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{54A44CBC-9319-4D71-856F-06858D6F8778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{970CE6BD-871F-4D74-BB1C-FA53DE68666A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Encabezado" sheetId="1" r:id="rId1"/>
@@ -73,7 +73,7 @@
     <t>Código de Barras</t>
   </si>
   <si>
-    <t>Código de Cirugía</t>
+    <t>Codigo de Cirugia</t>
   </si>
 </sst>
 </file>
@@ -465,15 +465,15 @@
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <f ca="1">TODAY()</f>
-        <v>45838</v>
+        <v>45881</v>
       </c>
       <c r="B2" s="1">
         <f ca="1">TODAY()</f>
-        <v>45838</v>
+        <v>45881</v>
       </c>
       <c r="G2" s="1">
         <f ca="1">TODAY()</f>
-        <v>45838</v>
+        <v>45881</v>
       </c>
       <c r="H2" s="3"/>
     </row>

</xml_diff>